<commit_message>
VMRSCode and empty description rows
</commit_message>
<xml_diff>
--- a/Rhubarb_7_1_B.xlsx
+++ b/Rhubarb_7_1_B.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" tabRatio="809"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" tabRatio="809" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Header" sheetId="2" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1492" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1494" uniqueCount="493">
   <si>
     <t>UP</t>
   </si>
@@ -1518,6 +1518,9 @@
   </si>
   <si>
     <t>234567</t>
+  </si>
+  <si>
+    <t>987123654</t>
   </si>
 </sst>
 </file>
@@ -6089,7 +6092,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X8"/>
+  <dimension ref="A1:Y8"/>
   <sheetFormatPr defaultColWidth="11.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
@@ -6111,13 +6114,14 @@
     <col min="18" max="18" width="26.85546875" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="30.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="34" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="25.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.28515625" style="1" customWidth="1"/>
+    <col min="22" max="22" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="30.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="34" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="25.140625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
         <v>8</v>
       </c>
@@ -6179,19 +6183,22 @@
         <v>140</v>
       </c>
       <c r="U1" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="V1" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="V1" s="18" t="s">
+      <c r="W1" s="18" t="s">
         <v>484</v>
       </c>
-      <c r="W1" s="18" t="s">
+      <c r="X1" s="18" t="s">
         <v>485</v>
       </c>
-      <c r="X1" s="18" t="s">
+      <c r="Y1" s="18" t="s">
         <v>488</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>182</v>
       </c>
@@ -6239,8 +6246,9 @@
       <c r="R2" s="3"/>
       <c r="S2" s="3"/>
       <c r="T2" s="4"/>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="U2" s="4"/>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>183</v>
       </c>
@@ -6288,8 +6296,9 @@
       <c r="R3" s="3"/>
       <c r="S3" s="3"/>
       <c r="T3" s="4"/>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="U3" s="4"/>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>184</v>
       </c>
@@ -6350,20 +6359,23 @@
       <c r="T4" s="4" t="s">
         <v>490</v>
       </c>
-      <c r="U4" s="1" t="s">
+      <c r="U4" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="V4" s="1" t="s">
         <v>489</v>
       </c>
-      <c r="V4" s="1" t="s">
+      <c r="W4" s="1" t="s">
         <v>486</v>
       </c>
-      <c r="W4" s="1" t="s">
+      <c r="X4" s="1" t="s">
         <v>487</v>
       </c>
-      <c r="X4" s="1" t="s">
+      <c r="Y4" s="1" t="s">
         <v>491</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>185</v>
       </c>
@@ -6411,8 +6423,9 @@
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
       <c r="T5" s="4"/>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="U5" s="4"/>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>456</v>
       </c>
@@ -6460,8 +6473,9 @@
       <c r="R6" s="3"/>
       <c r="S6" s="3"/>
       <c r="T6" s="4"/>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="U6" s="4"/>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>186</v>
       </c>
@@ -6509,8 +6523,9 @@
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
       <c r="T7" s="4"/>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="U7" s="4"/>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>187</v>
       </c>
@@ -6558,6 +6573,7 @@
       <c r="R8" s="3"/>
       <c r="S8" s="3"/>
       <c r="T8" s="4"/>
+      <c r="U8" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Language code optional, added INV
</commit_message>
<xml_diff>
--- a/Rhubarb_7_1_B.xlsx
+++ b/Rhubarb_7_1_B.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1494" uniqueCount="494">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1498" uniqueCount="496">
   <si>
     <t>UP</t>
   </si>
@@ -1524,6 +1524,12 @@
   </si>
   <si>
     <t>VMRSCode</t>
+  </si>
+  <si>
+    <t>Air Filter</t>
+  </si>
+  <si>
+    <t>INV</t>
   </si>
 </sst>
 </file>
@@ -6586,7 +6592,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
@@ -6606,7 +6612,7 @@
       <c r="C1" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="13" t="s">
         <v>48</v>
       </c>
       <c r="E1" s="19" t="s">
@@ -6634,14 +6640,14 @@
       <c r="A3" t="s">
         <v>182</v>
       </c>
-      <c r="B3" s="34" t="s">
-        <v>411</v>
+      <c r="B3" s="2" t="s">
+        <v>494</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>53</v>
+        <v>495</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>413</v>
+        <v>52</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -6649,16 +6655,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>183</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>412</v>
+        <v>182</v>
+      </c>
+      <c r="B4" s="34" t="s">
+        <v>411</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>53</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>52</v>
+        <v>413</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -6668,14 +6674,14 @@
       <c r="A5" t="s">
         <v>183</v>
       </c>
-      <c r="B5" s="34" t="s">
-        <v>411</v>
+      <c r="B5" s="2" t="s">
+        <v>412</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>53</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>413</v>
+        <v>52</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -6683,16 +6689,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>184</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>412</v>
+        <v>183</v>
+      </c>
+      <c r="B6" s="34" t="s">
+        <v>411</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>53</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>52</v>
+        <v>413</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -6702,14 +6708,14 @@
       <c r="A7" t="s">
         <v>184</v>
       </c>
-      <c r="B7" s="34" t="s">
-        <v>411</v>
+      <c r="B7" s="2" t="s">
+        <v>412</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>53</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>413</v>
+        <v>52</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -6717,16 +6723,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>456</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>457</v>
+        <v>184</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>411</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>53</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>52</v>
+        <v>413</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -6736,14 +6742,14 @@
       <c r="A9" t="s">
         <v>456</v>
       </c>
-      <c r="B9" s="34" t="s">
-        <v>458</v>
+      <c r="B9" s="2" t="s">
+        <v>457</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>53</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>413</v>
+        <v>52</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -6751,16 +6757,16 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>186</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>412</v>
+        <v>456</v>
+      </c>
+      <c r="B10" s="34" t="s">
+        <v>458</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>53</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>52</v>
+        <v>413</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -6770,14 +6776,14 @@
       <c r="A11" t="s">
         <v>186</v>
       </c>
-      <c r="B11" s="34" t="s">
-        <v>411</v>
+      <c r="B11" s="2" t="s">
+        <v>412</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>53</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>413</v>
+        <v>52</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -6785,16 +6791,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>187</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>412</v>
+        <v>186</v>
+      </c>
+      <c r="B12" s="34" t="s">
+        <v>411</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>53</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>52</v>
+        <v>413</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -6804,16 +6810,33 @@
       <c r="A13" t="s">
         <v>187</v>
       </c>
-      <c r="B13" s="34" t="s">
-        <v>411</v>
+      <c r="B13" s="2" t="s">
+        <v>412</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>53</v>
       </c>
       <c r="D13" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>187</v>
+      </c>
+      <c r="B14" s="34" t="s">
+        <v>411</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="E13">
+      <c r="E14">
         <v>1</v>
       </c>
     </row>

</xml_diff>